<commit_message>
plik z etykietami suwaka
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95558A36-8EFD-485B-BB2B-98C05D2DAB8F}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55356BF9-FCAB-4B6E-AB4E-FB41960A1537}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1044" yWindow="1236" windowWidth="11472" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,57 +25,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="13">
   <si>
     <t>image_path</t>
   </si>
   <si>
-    <t>label</t>
+    <t>label_text</t>
+  </si>
+  <si>
+    <t>left_label</t>
+  </si>
+  <si>
+    <t>right_label</t>
   </si>
   <si>
     <t>show_label</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\360_F_268212419_ZBJvlgVezhjziaP9aynnMGMLOvjUgNG5.jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\dachshund-8910099_640.jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\ee7bd76502e1d9aea7c74fc5bea75be9.jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (1).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (2).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (3).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (4).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (5).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images (6).jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\images.jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\istockphoto-1328935360-612x612.jpg</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\pexels-svetozar-milashevich-99573-1490908.jpg</t>
-  </si>
-  <si>
-    <t>Ten piesek jest smutny</t>
-  </si>
-  <si>
-    <t>Ten piesek jest wesoły</t>
+    <t>radość</t>
+  </si>
+  <si>
+    <t>smutek</t>
+  </si>
+  <si>
+    <t>strach</t>
+  </si>
+  <si>
+    <t>złość</t>
+  </si>
+  <si>
+    <t>zaufanie</t>
+  </si>
+  <si>
+    <t>wstręt</t>
+  </si>
+  <si>
+    <t>zaskoczenie</t>
+  </si>
+  <si>
+    <t>oczekiwanie</t>
   </si>
 </sst>
 </file>
@@ -393,15 +381,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="102.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -411,137 +401,267 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
poprawne aktualizowanie labeli z excela
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384CA377-8592-4A64-B0BC-E6945F425D5F}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E57CE29-66FD-441F-9FAC-9ED3168697A5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,9 +30,6 @@
     <t>image_path</t>
   </si>
   <si>
-    <t>label_text</t>
-  </si>
-  <si>
     <t>left_label</t>
   </si>
   <si>
@@ -70,6 +67,9 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>etykieta</t>
   </si>
 </sst>
 </file>
@@ -406,30 +406,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -437,16 +437,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -454,16 +454,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -471,16 +471,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
         <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -488,16 +488,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
         <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -505,16 +505,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
         <v>7</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -522,16 +522,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
         <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>10</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -539,16 +539,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
         <v>11</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -556,16 +556,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
         <v>5</v>
-      </c>
-      <c r="D10" t="s">
-        <v>6</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -573,16 +573,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
         <v>7</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -590,16 +590,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
         <v>9</v>
-      </c>
-      <c r="D12" t="s">
-        <v>10</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -607,16 +607,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" t="s">
         <v>11</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -624,16 +624,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
         <v>5</v>
-      </c>
-      <c r="D14" t="s">
-        <v>6</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -641,16 +641,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" t="s">
         <v>7</v>
-      </c>
-      <c r="D15" t="s">
-        <v>8</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -658,16 +658,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
         <v>9</v>
-      </c>
-      <c r="D16" t="s">
-        <v>10</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -675,16 +675,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" t="s">
         <v>11</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -692,16 +692,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
         <v>7</v>
-      </c>
-      <c r="D18" t="s">
-        <v>8</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -709,16 +709,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" t="s">
         <v>5</v>
-      </c>
-      <c r="D19" t="s">
-        <v>6</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -726,16 +726,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
         <v>11</v>
-      </c>
-      <c r="D20" t="s">
-        <v>12</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -743,16 +743,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
         <v>9</v>
-      </c>
-      <c r="D21" t="s">
-        <v>10</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -760,16 +760,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" t="s">
         <v>7</v>
-      </c>
-      <c r="D22" t="s">
-        <v>8</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -777,16 +777,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" t="s">
         <v>5</v>
-      </c>
-      <c r="D23" t="s">
-        <v>6</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -794,16 +794,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" t="s">
         <v>11</v>
-      </c>
-      <c r="D24" t="s">
-        <v>12</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -811,16 +811,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" t="s">
         <v>9</v>
-      </c>
-      <c r="D25" t="s">
-        <v>10</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -828,16 +828,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" t="s">
         <v>11</v>
-      </c>
-      <c r="D26" t="s">
-        <v>12</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -845,16 +845,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
         <v>9</v>
-      </c>
-      <c r="D27" t="s">
-        <v>10</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -862,16 +862,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" t="s">
         <v>7</v>
-      </c>
-      <c r="D28" t="s">
-        <v>8</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -879,16 +879,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" t="s">
         <v>5</v>
-      </c>
-      <c r="D29" t="s">
-        <v>6</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -896,16 +896,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" t="s">
         <v>11</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -913,16 +913,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
         <v>9</v>
-      </c>
-      <c r="D31" t="s">
-        <v>10</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -930,16 +930,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" t="s">
         <v>7</v>
-      </c>
-      <c r="D32" t="s">
-        <v>8</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -947,16 +947,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" t="s">
         <v>5</v>
-      </c>
-      <c r="D33" t="s">
-        <v>6</v>
       </c>
       <c r="E33">
         <v>1</v>

</xml_diff>

<commit_message>
drobne zmiany w excelu
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E57CE29-66FD-441F-9FAC-9ED3168697A5}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51AA7CE1-BEDD-44EE-A232-490F2F6FF3EB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="38">
   <si>
     <t>image_path</t>
   </si>
@@ -70,18 +70,95 @@
   </si>
   <si>
     <t>etykieta</t>
+  </si>
+  <si>
+    <t>warunek</t>
+  </si>
+  <si>
+    <t>sugestia</t>
+  </si>
+  <si>
+    <t>zgodny</t>
+  </si>
+  <si>
+    <t>proporcja</t>
+  </si>
+  <si>
+    <t>50/50</t>
+  </si>
+  <si>
+    <t>80/20 (strach)</t>
+  </si>
+  <si>
+    <t>80/20 (zaskoczenie)</t>
+  </si>
+  <si>
+    <t>80/20 (radość)</t>
+  </si>
+  <si>
+    <t>80/20 (zaufanie)</t>
+  </si>
+  <si>
+    <t>80/20 (Smutek)</t>
+  </si>
+  <si>
+    <t>80/20 (Wstręt)</t>
+  </si>
+  <si>
+    <t>80/20 (Złość)</t>
+  </si>
+  <si>
+    <t>80/20 (Strach)</t>
+  </si>
+  <si>
+    <t>80/20 (Zaskocz.)</t>
+  </si>
+  <si>
+    <t>80/20 (Radość)</t>
+  </si>
+  <si>
+    <t>80/20 (Zaufanie)</t>
+  </si>
+  <si>
+    <t>80/20 (Oczek.)</t>
+  </si>
+  <si>
+    <t>80/20 (oczek.)</t>
+  </si>
+  <si>
+    <t>kontrolny</t>
+  </si>
+  <si>
+    <t>niezgodny</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 80% radości.</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 75% zaufania.</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy strach.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -105,8 +182,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -391,17 +471,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="86.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -417,13 +498,19 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -434,13 +521,19 @@
       <c r="E2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -451,13 +544,19 @@
       <c r="E3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
@@ -468,13 +567,16 @@
       <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -485,8 +587,14 @@
       <c r="E5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -502,8 +610,14 @@
       <c r="E6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -519,8 +633,14 @@
       <c r="E7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -536,8 +656,14 @@
       <c r="E8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -553,13 +679,16 @@
       <c r="E9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>13</v>
       </c>
       <c r="C10" t="s">
         <v>4</v>
@@ -570,8 +699,14 @@
       <c r="E10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -587,8 +722,14 @@
       <c r="E11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -604,8 +745,14 @@
       <c r="E12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -621,8 +768,14 @@
       <c r="E13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -638,8 +791,14 @@
       <c r="E14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -655,8 +814,14 @@
       <c r="E15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -672,8 +837,14 @@
       <c r="E16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -689,8 +860,14 @@
       <c r="E17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -706,8 +883,14 @@
       <c r="E18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -723,8 +906,14 @@
       <c r="E19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -740,8 +929,14 @@
       <c r="E20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -757,8 +952,14 @@
       <c r="E21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -774,13 +975,16 @@
       <c r="E22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>12</v>
-      </c>
-      <c r="B23" t="s">
-        <v>13</v>
       </c>
       <c r="C23" t="s">
         <v>4</v>
@@ -791,8 +995,14 @@
       <c r="E23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -808,8 +1018,14 @@
       <c r="E24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -825,8 +1041,14 @@
       <c r="E25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -842,8 +1064,14 @@
       <c r="E26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -859,8 +1087,14 @@
       <c r="E27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -876,8 +1110,14 @@
       <c r="E28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -893,8 +1133,14 @@
       <c r="E29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -910,13 +1156,16 @@
       <c r="E30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>12</v>
-      </c>
-      <c r="B31" t="s">
-        <v>13</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
@@ -927,8 +1176,14 @@
       <c r="E31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -944,8 +1199,14 @@
       <c r="E32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -960,6 +1221,12 @@
       </c>
       <c r="E33">
         <v>1</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G33" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prawdopodobnie finalna wersja excela
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="402" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EE544A9-44E3-4CE5-AFEF-A3931A489517}"/>
+  <xr:revisionPtr revIDLastSave="484" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACE548B4-62A4-4341-9516-64552FBE22A6}"/>
   <bookViews>
-    <workbookView xWindow="10212" yWindow="0" windowWidth="12924" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="102">
   <si>
     <t>image_path</t>
   </si>
@@ -63,9 +63,6 @@
     <t>oczekiwanie</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\ee7bd76502e1d9aea7c74fc5bea75be9.jpg</t>
-  </si>
-  <si>
     <t>etykieta</t>
   </si>
   <si>
@@ -81,15 +78,6 @@
     <t>Poprzedni badani wykryli w tej twarzy strach.</t>
   </si>
   <si>
-    <t xml:space="preserve">80/20 </t>
-  </si>
-  <si>
-    <t>80/20</t>
-  </si>
-  <si>
-    <t>dominacja/kierunek</t>
-  </si>
-  <si>
     <t>n/d</t>
   </si>
   <si>
@@ -171,15 +159,9 @@
     <t>Kategorialna AI</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy % .</t>
-  </si>
-  <si>
     <t>kontrolna</t>
   </si>
   <si>
-    <t>Poprzedni badani wykryli w tej twarzy % .</t>
-  </si>
-  <si>
     <t>Poprzedni badani wykryli w tej twarzy oczekiwanie.</t>
   </si>
   <si>
@@ -192,9 +174,6 @@
     <t>Model sztucznej inteligencji wykrył w tej twarzy zaskoczenie.</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 80% złości.</t>
-  </si>
-  <si>
     <t>Model sztucznej inteligencji wykrył w tej twarzy strach.</t>
   </si>
   <si>
@@ -213,21 +192,9 @@
     <t>Poprzedni badani wykryli w tej twarzy 20% zaufania.</t>
   </si>
   <si>
-    <t>80/20 (wstręt)</t>
-  </si>
-  <si>
-    <t>proporcja_zdjęcia</t>
-  </si>
-  <si>
     <t>typ_etykiety</t>
   </si>
   <si>
-    <t>80/20 prawo</t>
-  </si>
-  <si>
-    <t>80/20 lewo</t>
-  </si>
-  <si>
     <t>80/20 oczekiwanie</t>
   </si>
   <si>
@@ -240,31 +207,150 @@
     <t>80/20 smutek</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 74% smutku .</t>
-  </si>
-  <si>
-    <t>Poprzedni badani wykryli w tej twarzy 83% zaufania.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 81% zaufania .</t>
-  </si>
-  <si>
-    <t>Poprzedni badani wykryli w tej twarzy 79% smutku.</t>
-  </si>
-  <si>
-    <t>Poprzedni badani wykryli w tej twarzy 80% oczekiwania.</t>
+    <t>80/20 zaufania</t>
+  </si>
+  <si>
+    <t>80/20 złość</t>
+  </si>
+  <si>
+    <t>80/20 zaskoczenie</t>
+  </si>
+  <si>
+    <t>80/20 wstręt</t>
+  </si>
+  <si>
+    <t>80/20 zaufanie</t>
+  </si>
+  <si>
+    <t>80/20 strach</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\1K SZ 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\1M SZ 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\2K SZ 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\2M SZ 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\1K RS 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\1M RS 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\2K RS 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\2M RS 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\1K ZO 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\1M ZO 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\2K ZO 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\2M ZO 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\1K ZW 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\1M ZW 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\2K ZW 5050.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\2M ZW 5050.png</t>
+  </si>
+  <si>
+    <t>proporcja_zdjecia</t>
+  </si>
+  <si>
+    <t>kierunek</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 79% smutku.</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 23% smutku.</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 95% zaufania.</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 78% zaufania.</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 21% zaskoczenia.</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 19% złości.</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\OZ 80,20\1K OZ 8020.png</t>
+  </si>
+  <si>
+    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\OZ 80,20\1M OZ 8020.png</t>
+  </si>
+  <si>
+    <t>80/20 lewo (zaskoczenie)</t>
+  </si>
+  <si>
+    <t>80/20 prawo (złość)</t>
+  </si>
+  <si>
+    <t>80/20 radość</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy smutek.</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 75% oczekiwania.</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 78% smutku.</t>
+  </si>
+  <si>
+    <t>80/20 lewo (radość)</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 81% zaufania.</t>
+  </si>
+  <si>
+    <t>80/20 prawo (wstręt)</t>
+  </si>
+  <si>
+    <t>Poprzedni badani wykryli w tej twarzy 92% oczekiwania.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -329,28 +415,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -641,14 +730,14 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="86.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.44140625" customWidth="1"/>
-    <col min="6" max="6" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" customWidth="1"/>
     <col min="7" max="7" width="17.21875" customWidth="1"/>
     <col min="8" max="8" width="11.109375" customWidth="1"/>
-    <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -656,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -668,24 +757,24 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="G1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -697,24 +786,24 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -726,24 +815,24 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -755,24 +844,21 @@
         <v>0</v>
       </c>
       <c r="F4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="I4" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -784,24 +870,24 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -813,24 +899,21 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -842,24 +925,24 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
@@ -871,24 +954,21 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -900,24 +980,24 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
@@ -929,24 +1009,21 @@
         <v>1</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -957,25 +1034,25 @@
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>19</v>
+      <c r="F11" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -987,24 +1064,24 @@
         <v>1</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -1016,24 +1093,21 @@
         <v>0</v>
       </c>
       <c r="F13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="I13" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -1044,25 +1118,25 @@
       <c r="E14">
         <v>1</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="I14" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
@@ -1074,24 +1148,21 @@
         <v>1</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
         <v>44</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" t="s">
-        <v>49</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -1103,24 +1174,21 @@
         <v>0</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>12</v>
-      </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
@@ -1131,25 +1199,25 @@
       <c r="E17">
         <v>1</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>22</v>
-      </c>
       <c r="I17" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
         <v>4</v>
@@ -1161,24 +1229,24 @@
         <v>1</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
         <v>10</v>
@@ -1190,24 +1258,24 @@
         <v>0</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1219,24 +1287,21 @@
         <v>1</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>12</v>
-      </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
         <v>6</v>
@@ -1247,25 +1312,22 @@
       <c r="E21">
         <v>1</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>19</v>
+      <c r="F21" s="9" t="s">
+        <v>61</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>12</v>
-      </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1276,25 +1338,25 @@
       <c r="E22">
         <v>1</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>19</v>
+      <c r="F22" s="9" t="s">
+        <v>64</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
         <v>10</v>
@@ -1306,24 +1368,21 @@
         <v>0</v>
       </c>
       <c r="F23" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="I23" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>12</v>
-      </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="C24" t="s">
         <v>4</v>
@@ -1334,25 +1393,25 @@
       <c r="E24">
         <v>1</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="I24" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1364,24 +1423,24 @@
         <v>1</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
@@ -1393,24 +1452,21 @@
         <v>1</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>12</v>
-      </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
@@ -1421,25 +1477,25 @@
       <c r="E27">
         <v>1</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>19</v>
+      <c r="F27" s="9" t="s">
+        <v>65</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
         <v>10</v>
@@ -1451,24 +1507,21 @@
         <v>1</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
         <v>44</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B29" t="s">
-        <v>49</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
@@ -1480,24 +1533,24 @@
         <v>0</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="B30" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C30" t="s">
         <v>4</v>
@@ -1509,24 +1562,21 @@
         <v>1</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>12</v>
-      </c>
       <c r="B31" t="s">
-        <v>50</v>
+        <v>101</v>
       </c>
       <c r="C31" t="s">
         <v>10</v>
@@ -1537,25 +1587,25 @@
       <c r="E31">
         <v>1</v>
       </c>
-      <c r="F31" s="3" t="s">
-        <v>19</v>
+      <c r="F31" s="9" t="s">
+        <v>56</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1567,24 +1617,21 @@
         <v>0</v>
       </c>
       <c r="F32" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H32" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H32" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="I32" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>12</v>
-      </c>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C33" t="s">
         <v>4</v>
@@ -1596,16 +1643,16 @@
         <v>1</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
zamiana sciezki lokalnej na globalna
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="553" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C2FF190-E086-463E-B9AF-EFAB3FB3BE3B}"/>
+  <xr:revisionPtr revIDLastSave="638" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BB2EF89-10C8-4920-B568-53A7614C1AF0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,54 +219,6 @@
     <t>80/20 strach</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\1K SZ 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\1M SZ 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\2K SZ 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\SZ 50,50\2M SZ 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\1K RS 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\1M RS 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\2K RS 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\RS 50,50\2M RS 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\1K ZO 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\1M ZO 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\2K ZO 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZO 50,50\2M ZO 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\1K ZW 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\1M ZW 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\2K ZW 5050.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 50,50\ZW 50,50\2M ZW 5050.png</t>
-  </si>
-  <si>
     <t>proporcja_zdjecia</t>
   </si>
   <si>
@@ -291,12 +243,6 @@
     <t>Model sztucznej inteligencji wykrył w tej twarzy 19% złości.</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\OZ 80,20\1K OZ 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\OZ 80,20\1M OZ 8020.png</t>
-  </si>
-  <si>
     <t>80/20 lewo (zaskoczenie)</t>
   </si>
   <si>
@@ -327,46 +273,100 @@
     <t>Poprzedni badani wykryli w tej twarzy 92% oczekiwania.</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\RS 80,20\1K RS 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\RS 80,20\1M RS 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\SR 80,20\1K SR 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\SR 80,20\1M SR 8020.png</t>
-  </si>
-  <si>
     <t>Dominacja lewo strach</t>
   </si>
   <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\SZ 80,20\1K SZ 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\SZ 80,20\1M SZ 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\ZS 80,20\1K ZS 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\ZS 80,20\1M ZS 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\WZ 80,20\1K WZ 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\WZ 80,20\1M WZ 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\ZW 80,20\1K ZW 8020.png</t>
-  </si>
-  <si>
-    <t>C:\Users\julia\OneDrive\Pulpit\percepcja_psychopy\photos\Twarze 80,20\ZW 80,20\1M ZW 8020.png</t>
-  </si>
-  <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>photos\1K_SZ_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_OZ_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1K_RS_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_ZW_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1M_SR_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1K_ZO_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_ZS_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1K_ZW_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_RS_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1M_ZO_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_ZS_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1M_RS_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_ZW_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_SZ_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_RS_8020.png</t>
+  </si>
+  <si>
+    <t>photos\1K_WZ_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2K_RS_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_ZW_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2K_ZW_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_SZ_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2M_SZ_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_OZ_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2M_RS_5050.png</t>
+  </si>
+  <si>
+    <t>photos\2K_ZO_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1K_SR_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2K_SZ_5050.png</t>
+  </si>
+  <si>
+    <t>photos\2M_ZW_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_SZ_8020.png</t>
+  </si>
+  <si>
+    <t>photos\2M_ZO_5050.png</t>
+  </si>
+  <si>
+    <t>photos\1M_WZ_8020.png</t>
   </si>
 </sst>
 </file>
@@ -804,7 +804,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="G1" t="s">
         <v>53</v>
@@ -813,12 +813,12 @@
         <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
@@ -847,7 +847,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
         <v>44</v>
@@ -876,10 +876,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -905,7 +905,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>52</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -963,10 +963,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -978,7 +978,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>41</v>
@@ -992,7 +992,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
         <v>45</v>
@@ -1021,10 +1021,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -1036,7 +1036,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>43</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
         <v>47</v>
@@ -1079,10 +1079,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -1108,10 +1108,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="B13" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -1166,10 +1166,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -1195,7 +1195,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -1239,7 +1239,7 @@
         <v>4</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>41</v>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
         <v>50</v>
@@ -1282,7 +1282,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
@@ -1311,10 +1311,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C19" t="s">
         <v>10</v>
@@ -1326,7 +1326,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>41</v>
@@ -1340,10 +1340,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B21" t="s">
         <v>16</v>
@@ -1393,15 +1393,15 @@
         <v>18</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1427,10 +1427,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
         <v>10</v>
@@ -1456,10 +1456,10 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="C24" t="s">
         <v>4</v>
@@ -1485,7 +1485,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="B25" t="s">
         <v>49</v>
@@ -1514,10 +1514,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" t="s">
         <v>79</v>
-      </c>
-      <c r="B26" t="s">
-        <v>97</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
@@ -1543,7 +1543,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B27" t="s">
         <v>48</v>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="B28" t="s">
         <v>44</v>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
@@ -1616,7 +1616,7 @@
         <v>4</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>41</v>
@@ -1630,10 +1630,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="B30" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
         <v>4</v>
@@ -1659,10 +1659,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="B31" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="C31" t="s">
         <v>10</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1717,7 +1717,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B33" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
finalna wersja!!!1!! plus zamiana nazwy
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="639" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7239576F-B65A-46C2-BAB1-3CBE66757D8C}"/>
+  <xr:revisionPtr revIDLastSave="645" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20511CCC-87FE-461C-B167-1ABF936BEAE3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -180,9 +180,6 @@
     <t>Model sztucznej inteligencji wykrył w tej twarzy wstręt.</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 72% strachu .</t>
-  </si>
-  <si>
     <t>Poprzedni badani wykryli w tej twarzy 20% zaufania.</t>
   </si>
   <si>
@@ -367,6 +364,9 @@
   </si>
   <si>
     <t>photos/1M_SR_8020.png</t>
+  </si>
+  <si>
+    <t>Model sztucznej inteligencji wykrył w tej twarzy 72% strachu.</t>
   </si>
 </sst>
 </file>
@@ -804,24 +804,24 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H1" t="s">
         <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -847,7 +847,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
         <v>44</v>
@@ -862,7 +862,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>40</v>
@@ -876,10 +876,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -905,10 +905,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>42</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -949,7 +949,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>42</v>
@@ -963,10 +963,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -978,7 +978,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>41</v>
@@ -992,7 +992,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
         <v>45</v>
@@ -1021,10 +1021,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -1036,7 +1036,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>43</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B10" t="s">
         <v>47</v>
@@ -1079,10 +1079,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -1094,7 +1094,7 @@
         <v>4</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>39</v>
@@ -1108,10 +1108,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -1166,10 +1166,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -1181,7 +1181,7 @@
         <v>4</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>39</v>
@@ -1195,7 +1195,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -1236,10 +1236,10 @@
         <v>5</v>
       </c>
       <c r="E16">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>41</v>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
         <v>50</v>
@@ -1268,7 +1268,7 @@
         <v>4</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>43</v>
@@ -1282,7 +1282,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
@@ -1311,10 +1311,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
         <v>10</v>
@@ -1323,10 +1323,10 @@
         <v>11</v>
       </c>
       <c r="E19">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>41</v>
@@ -1340,10 +1340,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B21" t="s">
         <v>16</v>
@@ -1384,7 +1384,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>40</v>
@@ -1393,15 +1393,15 @@
         <v>18</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1413,7 +1413,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>42</v>
@@ -1427,10 +1427,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
         <v>10</v>
@@ -1439,7 +1439,7 @@
         <v>11</v>
       </c>
       <c r="E23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>14</v>
@@ -1456,10 +1456,10 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C24" t="s">
         <v>4</v>
@@ -1471,7 +1471,7 @@
         <v>4</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>39</v>
@@ -1485,7 +1485,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B25" t="s">
         <v>49</v>
@@ -1514,10 +1514,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
@@ -1543,7 +1543,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" t="s">
         <v>48</v>
@@ -1558,7 +1558,7 @@
         <v>4</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>43</v>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
         <v>44</v>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
@@ -1613,10 +1613,10 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>41</v>
@@ -1630,10 +1630,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
         <v>4</v>
@@ -1659,10 +1659,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
         <v>10</v>
@@ -1674,7 +1674,7 @@
         <v>4</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>42</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1700,7 +1700,7 @@
         <v>7</v>
       </c>
       <c r="E32">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>14</v>
@@ -1717,10 +1717,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C33" t="s">
         <v>4</v>
@@ -1732,7 +1732,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
finalna wersja i finalny kod js
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="645" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20511CCC-87FE-461C-B167-1ABF936BEAE3}"/>
+  <xr:revisionPtr revIDLastSave="647" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4617873-AF3E-4610-A354-76C5CAC217D9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="116">
   <si>
     <t>image_path</t>
   </si>
@@ -367,6 +367,12 @@
   </si>
   <si>
     <t>Model sztucznej inteligencji wykrył w tej twarzy 72% strachu.</t>
+  </si>
+  <si>
+    <t>photos/1K_ZO_8020.png</t>
+  </si>
+  <si>
+    <t>photos/1M_ZO_8020.png</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1172,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="B14" t="s">
         <v>69</v>
@@ -1311,7 +1317,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
zamiana si na ai
</commit_message>
<xml_diff>
--- a/conditions.xlsx
+++ b/conditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6412cbcd551681e8/Pulpit/percepcja_psychopy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="647" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4617873-AF3E-4610-A354-76C5CAC217D9}"/>
+  <xr:revisionPtr revIDLastSave="648" documentId="11_F25DC773A252ABDACC104859311E590A5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5D380BF-963F-468A-A529-3EAAE1FB28AE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,21 +165,6 @@
     <t>Poprzedni badani wykryli w tej twarzy wstręt.</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy radość.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy zaskoczenie.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy strach.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy złość.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy wstręt.</t>
-  </si>
-  <si>
     <t>Poprzedni badani wykryli w tej twarzy 20% zaufania.</t>
   </si>
   <si>
@@ -222,24 +207,9 @@
     <t>kierunek</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 79% smutku.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 23% smutku.</t>
-  </si>
-  <si>
     <t>Poprzedni badani wykryli w tej twarzy 95% zaufania.</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 78% zaufania.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 21% zaskoczenia.</t>
-  </si>
-  <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 19% złości.</t>
-  </si>
-  <si>
     <t>80/20 lewo (zaskoczenie)</t>
   </si>
   <si>
@@ -249,9 +219,6 @@
     <t>80/20 radość</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy smutek.</t>
-  </si>
-  <si>
     <t>Poprzedni badani wykryli w tej twarzy 75% oczekiwania.</t>
   </si>
   <si>
@@ -366,13 +333,46 @@
     <t>photos/1M_SR_8020.png</t>
   </si>
   <si>
-    <t>Model sztucznej inteligencji wykrył w tej twarzy 72% strachu.</t>
-  </si>
-  <si>
     <t>photos/1K_ZO_8020.png</t>
   </si>
   <si>
     <t>photos/1M_ZO_8020.png</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 72% strachu.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy smutek.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy zaskoczenie.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 19% złości.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 21% zaskoczenia.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy wstręt.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy radość.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 78% zaufania.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 23% smutku.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy złość.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy strach.</t>
+  </si>
+  <si>
+    <t>Model AI wykrył w tej twarzy 79% smutku.</t>
   </si>
 </sst>
 </file>
@@ -810,24 +810,24 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H1" t="s">
         <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -853,7 +853,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
         <v>44</v>
@@ -868,7 +868,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>40</v>
@@ -882,10 +882,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -911,10 +911,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -926,7 +926,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>42</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -955,7 +955,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>42</v>
@@ -969,10 +969,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>41</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
         <v>45</v>
@@ -1027,10 +1027,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -1042,7 +1042,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>43</v>
@@ -1056,10 +1056,10 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
@@ -1085,10 +1085,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -1100,7 +1100,7 @@
         <v>4</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>39</v>
@@ -1114,10 +1114,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
@@ -1143,10 +1143,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -1172,10 +1172,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -1187,7 +1187,7 @@
         <v>4</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>39</v>
@@ -1201,7 +1201,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1230,10 +1230,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -1245,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>41</v>
@@ -1259,10 +1259,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
@@ -1274,7 +1274,7 @@
         <v>4</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>43</v>
@@ -1288,10 +1288,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="C18" t="s">
         <v>4</v>
@@ -1317,10 +1317,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
         <v>10</v>
@@ -1332,7 +1332,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>41</v>
@@ -1346,10 +1346,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
         <v>16</v>
@@ -1390,7 +1390,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>40</v>
@@ -1399,15 +1399,15 @@
         <v>18</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1419,7 +1419,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>42</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>10</v>
@@ -1462,10 +1462,10 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
         <v>4</v>
@@ -1477,7 +1477,7 @@
         <v>4</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>39</v>
@@ -1491,10 +1491,10 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1520,10 +1520,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
@@ -1549,10 +1549,10 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
@@ -1564,7 +1564,7 @@
         <v>4</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>43</v>
@@ -1578,7 +1578,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="B28" t="s">
         <v>44</v>
@@ -1607,10 +1607,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B29" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>41</v>
@@ -1636,10 +1636,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>115</v>
       </c>
       <c r="C30" t="s">
         <v>4</v>
@@ -1665,10 +1665,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C31" t="s">
         <v>10</v>
@@ -1680,7 +1680,7 @@
         <v>4</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>42</v>
@@ -1694,10 +1694,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1723,10 +1723,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B33" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C33" t="s">
         <v>4</v>
@@ -1738,7 +1738,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>40</v>

</xml_diff>